<commit_message>
Test DK weather file
</commit_message>
<xml_diff>
--- a/examples/building_input.xlsx
+++ b/examples/building_input.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://windowmaster-my.sharepoint.com/personal/aza_dk_windowmaster_com/Documents/99_Other/Documents/GitHub/pyBuildingEnergy/examples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="13_ncr:1_{D98B15CA-71BB-4E34-A4E0-6F07676CE52B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{76A6418D-F777-4802-A8B8-ECEE6D8EF907}"/>
+  <xr:revisionPtr revIDLastSave="31" documentId="13_ncr:1_{D98B15CA-71BB-4E34-A4E0-6F07676CE52B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B548F614-8621-41B1-9F55-8F96C82C94E0}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="30936" windowHeight="16776" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="30936" windowHeight="16776" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <sheet name="Profiles" sheetId="4" r:id="rId4"/>
     <sheet name="Summary" sheetId="5" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -5656,7 +5656,7 @@
         <v>57</v>
       </c>
       <c r="C15" s="4">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="D15" s="3" t="s">
         <v>58</v>
@@ -5673,7 +5673,7 @@
         <v>61</v>
       </c>
       <c r="C16" s="4">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D16" s="3" t="s">
         <v>62</v>
@@ -5688,7 +5688,7 @@
         <v>64</v>
       </c>
       <c r="C17" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D17" s="3" t="s">
         <v>31</v>
@@ -5924,7 +5924,7 @@
         <v>106</v>
       </c>
       <c r="C33" s="4">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D33" s="3" t="s">
         <v>102</v>
@@ -5967,7 +5967,7 @@
         <v>114</v>
       </c>
       <c r="C36" s="4">
-        <v>4.2</v>
+        <v>0</v>
       </c>
       <c r="D36" s="3" t="s">
         <v>115</v>
@@ -5999,7 +5999,7 @@
         <v>120</v>
       </c>
       <c r="C38" s="4">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D38" s="3" t="s">
         <v>115</v>
@@ -6230,10 +6230,10 @@
         <v>741500</v>
       </c>
       <c r="K6" s="4">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="L6" s="4">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="M6" s="5"/>
       <c r="N6" s="5"/>
@@ -6275,10 +6275,10 @@
         <v>1416240</v>
       </c>
       <c r="K7" s="4">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="L7" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M7" s="5"/>
       <c r="N7" s="5"/>
@@ -6320,10 +6320,10 @@
         <v>1416240</v>
       </c>
       <c r="K8" s="4">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="L8" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M8" s="5"/>
       <c r="N8" s="5"/>
@@ -6365,10 +6365,10 @@
         <v>1416240</v>
       </c>
       <c r="K9" s="4">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="L9" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M9" s="5"/>
       <c r="N9" s="5"/>
@@ -6410,10 +6410,10 @@
         <v>1416240</v>
       </c>
       <c r="K10" s="4">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="L10" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M10" s="5"/>
       <c r="N10" s="5"/>
@@ -6455,10 +6455,10 @@
         <v>405801</v>
       </c>
       <c r="K11" s="4">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="L11" s="4">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="M11" s="5"/>
       <c r="N11" s="5"/>
@@ -6500,7 +6500,7 @@
         <v>0</v>
       </c>
       <c r="K12" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="5">
@@ -6558,7 +6558,7 @@
         <v>0</v>
       </c>
       <c r="K13" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L13" s="4"/>
       <c r="M13" s="5">
@@ -8593,7 +8593,7 @@
       </c>
       <c r="B3" s="17">
         <f>Building!$C$15</f>
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>58</v>
@@ -8653,7 +8653,7 @@
       </c>
       <c r="B8" s="18">
         <f>IF(B3&gt;0,B6/B3,0)</f>
-        <v>6.6666666666666666E-2</v>
+        <v>0.08</v>
       </c>
       <c r="C8" s="3"/>
     </row>
@@ -8682,7 +8682,7 @@
       </c>
       <c r="B11" s="17">
         <f>Building!$C$33</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>102</v>
@@ -8694,7 +8694,7 @@
       </c>
       <c r="B12" s="17">
         <f>B10+B11</f>
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>102</v>
@@ -8718,7 +8718,7 @@
       </c>
       <c r="B14" s="17">
         <f>IF(B3&gt;0,B12/B3,0)</f>
-        <v>1.5833333333333333</v>
+        <v>1.88</v>
       </c>
       <c r="C14" s="3" t="s">
         <v>202</v>

</xml_diff>